<commit_message>
Add per-match points chart, team colours, home-page polish; fix name-match false positives
- Surname-gated matcher + dedupe stops a not-yet-played player (david willey)
  inheriting a different player's stats (david miller); Miller now scores only
  for ssw. All teams' per-match totals reconcile with season totals.
- New Match_Team_Points data + 'Points Gained Per Match' grouped-bar chart.
- Consistent per-team colours across all charts; leader card shows margin.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Hundred_Fantasy_Points.xlsx
+++ b/Hundred_Fantasy_Points.xlsx
@@ -13,6 +13,7 @@
     <sheet name="No_Stats_Yet" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Possible_Mismatch" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="AI_Matches" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Match_Team_Points" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4934,33 +4935,29 @@
       <c r="E62" t="b">
         <v>0</v>
       </c>
-      <c r="F62" t="inlineStr">
+      <c r="F62" t="inlineStr"/>
+      <c r="G62" t="inlineStr"/>
+      <c r="H62" t="inlineStr">
         <is>
           <t>david miller</t>
         </is>
       </c>
-      <c r="G62" t="inlineStr">
-        <is>
-          <t>David Miller</t>
-        </is>
-      </c>
-      <c r="H62" t="inlineStr"/>
       <c r="I62" t="inlineStr">
         <is>
-          <t>fuzzy_margin:83.33333333333334</t>
+          <t>no_stats_yet</t>
         </is>
       </c>
       <c r="J62" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K62" t="n">
-        <v>44</v>
+        <v>0</v>
       </c>
       <c r="L62" t="n">
         <v>0</v>
       </c>
       <c r="M62" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N62" t="n">
         <v>0</v>
@@ -4969,22 +4966,22 @@
         <v>0</v>
       </c>
       <c r="P62" t="n">
-        <v>54</v>
+        <v>0</v>
       </c>
       <c r="Q62" t="n">
         <v>0</v>
       </c>
       <c r="R62" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="S62" t="n">
-        <v>66</v>
+        <v>0</v>
       </c>
       <c r="T62" t="n">
         <v>1</v>
       </c>
       <c r="U62" t="n">
-        <v>66</v>
+        <v>0</v>
       </c>
     </row>
     <row r="63">
@@ -6448,7 +6445,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>222</v>
+        <v>156</v>
       </c>
     </row>
     <row r="6">
@@ -9021,7 +9018,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U44"/>
+  <dimension ref="A1:U45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11406,12 +11403,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>mitchell owen</t>
+          <t>david willey</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>ssw</t>
+          <t>lg</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -11429,7 +11426,7 @@
       <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr">
         <is>
-          <t>mitchell marsh</t>
+          <t>david miller</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -11477,12 +11474,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>craig overton</t>
+          <t>mitchell owen</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>cc</t>
+          <t>ssw</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -11500,7 +11497,7 @@
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr">
         <is>
-          <t>chris jordan</t>
+          <t>mitchell marsh</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -11548,12 +11545,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>liam dawson</t>
+          <t>craig overton</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>lg</t>
+          <t>cc</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -11571,7 +11568,7 @@
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr">
         <is>
-          <t>tom alsop</t>
+          <t>chris jordan</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -11619,12 +11616,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>mitchell santner</t>
+          <t>liam dawson</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>cc</t>
+          <t>lg</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -11642,7 +11639,7 @@
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr">
         <is>
-          <t>mitchell marsh</t>
+          <t>tom alsop</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -11690,12 +11687,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>chris wood</t>
+          <t>mitchell santner</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>lg</t>
+          <t>cc</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -11713,7 +11710,7 @@
       <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr">
         <is>
-          <t>chris woakes</t>
+          <t>mitchell marsh</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -11761,12 +11758,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>gus atkinson</t>
+          <t>chris wood</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>f9</t>
+          <t>lg</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -11784,7 +11781,7 @@
       <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr">
         <is>
-          <t>marco jansen</t>
+          <t>chris woakes</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -11832,12 +11829,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>mustafizur rahman</t>
+          <t>gus atkinson</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>ssw</t>
+          <t>f9</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -11855,7 +11852,7 @@
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr">
         <is>
-          <t>sam curran</t>
+          <t>marco jansen</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -11903,12 +11900,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>saqib mahmood</t>
+          <t>mustafizur rahman</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>lg</t>
+          <t>ssw</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -11926,7 +11923,7 @@
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr">
         <is>
-          <t>abrar ahmed</t>
+          <t>sam curran</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -11974,7 +11971,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>reece topley</t>
+          <t>saqib mahmood</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -11997,7 +11994,7 @@
       <c r="G42" t="inlineStr"/>
       <c r="H42" t="inlineStr">
         <is>
-          <t>trent boult</t>
+          <t>abrar ahmed</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -12045,7 +12042,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>bradley currie</t>
+          <t>reece topley</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -12068,7 +12065,7 @@
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr">
         <is>
-          <t>brydon carse</t>
+          <t>trent boult</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -12116,12 +12113,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>matt henry</t>
+          <t>bradley currie</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>cc</t>
+          <t>lg</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -12139,48 +12136,119 @@
       <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr">
         <is>
+          <t>brydon carse</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>no_stats_yet</t>
+        </is>
+      </c>
+      <c r="J44" t="n">
+        <v>0</v>
+      </c>
+      <c r="K44" t="n">
+        <v>0</v>
+      </c>
+      <c r="L44" t="n">
+        <v>0</v>
+      </c>
+      <c r="M44" t="n">
+        <v>0</v>
+      </c>
+      <c r="N44" t="n">
+        <v>0</v>
+      </c>
+      <c r="O44" t="n">
+        <v>0</v>
+      </c>
+      <c r="P44" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q44" t="n">
+        <v>0</v>
+      </c>
+      <c r="R44" t="n">
+        <v>0</v>
+      </c>
+      <c r="S44" t="n">
+        <v>0</v>
+      </c>
+      <c r="T44" t="n">
+        <v>1</v>
+      </c>
+      <c r="U44" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>matt henry</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>cc</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>NAN</t>
+        </is>
+      </c>
+      <c r="D45" t="b">
+        <v>0</v>
+      </c>
+      <c r="E45" t="b">
+        <v>0</v>
+      </c>
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" t="inlineStr"/>
+      <c r="H45" t="inlineStr">
+        <is>
           <t>matthew short</t>
         </is>
       </c>
-      <c r="I44" t="inlineStr">
+      <c r="I45" t="inlineStr">
         <is>
           <t>no_stats_yet</t>
         </is>
       </c>
-      <c r="J44" t="n">
-        <v>0</v>
-      </c>
-      <c r="K44" t="n">
-        <v>0</v>
-      </c>
-      <c r="L44" t="n">
-        <v>0</v>
-      </c>
-      <c r="M44" t="n">
-        <v>0</v>
-      </c>
-      <c r="N44" t="n">
-        <v>0</v>
-      </c>
-      <c r="O44" t="n">
-        <v>0</v>
-      </c>
-      <c r="P44" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q44" t="n">
-        <v>0</v>
-      </c>
-      <c r="R44" t="n">
-        <v>0</v>
-      </c>
-      <c r="S44" t="n">
-        <v>0</v>
-      </c>
-      <c r="T44" t="n">
-        <v>1</v>
-      </c>
-      <c r="U44" t="n">
+      <c r="J45" t="n">
+        <v>0</v>
+      </c>
+      <c r="K45" t="n">
+        <v>0</v>
+      </c>
+      <c r="L45" t="n">
+        <v>0</v>
+      </c>
+      <c r="M45" t="n">
+        <v>0</v>
+      </c>
+      <c r="N45" t="n">
+        <v>0</v>
+      </c>
+      <c r="O45" t="n">
+        <v>0</v>
+      </c>
+      <c r="P45" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q45" t="n">
+        <v>0</v>
+      </c>
+      <c r="R45" t="n">
+        <v>0</v>
+      </c>
+      <c r="S45" t="n">
+        <v>0</v>
+      </c>
+      <c r="T45" t="n">
+        <v>1</v>
+      </c>
+      <c r="U45" t="n">
         <v>0</v>
       </c>
     </row>
@@ -12429,4 +12497,220 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>MatchNo</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Match</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Team</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>M1: MI London v Sunrisers Leeds</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>cc</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>M1: MI London v Sunrisers Leeds</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>f9</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>M1: MI London v Sunrisers Leeds</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>lg</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>M1: MI London v Sunrisers Leeds</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>sd</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>M1: MI London v Sunrisers Leeds</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>ssw</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>M2: Southern Brave v Welsh Fire</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>cc</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>2</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>M2: Southern Brave v Welsh Fire</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>f9</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>M2: Southern Brave v Welsh Fire</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>lg</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>2</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>M2: Southern Brave v Welsh Fire</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>sd</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>2</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>M2: Southern Brave v Welsh Fire</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>ssw</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>179</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>